<commit_message>
30 regions. fail cal 1990 cent asia dist heat fail solve 2065
</commit_message>
<xml_diff>
--- a/gcam-data-system/energy-data/assumptions/Tables_A20s.xlsx
+++ b/gcam-data-system/energy-data/assumptions/Tables_A20s.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="23416"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="32140" windowHeight="21340" tabRatio="684" firstSheet="43" activeTab="43"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="15960" tabRatio="684" firstSheet="26" activeTab="27"/>
   </bookViews>
   <sheets>
     <sheet name="A21.sector.csv" sheetId="5" r:id="rId1"/>
@@ -756,8 +756,22 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1685">
+  <cellStyleXfs count="1699">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -2451,7 +2465,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1685">
+  <cellStyles count="1699">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" hidden="1"/>
@@ -3294,6 +3308,13 @@
     <cellStyle name="Followed Hyperlink" xfId="1680" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="1682" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="1684" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="1686" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="1688" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="1690" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="1692" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="1694" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="1696" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="1698" builtinId="9" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="3" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="5" builtinId="8" hidden="1"/>
@@ -4136,6 +4157,13 @@
     <cellStyle name="Hyperlink" xfId="1679" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="1681" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="1683" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="1685" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="1687" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="1689" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="1691" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="1693" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="1695" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="1697" builtinId="8" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>

</xml_diff>

<commit_message>
corrected delivery costs for gas, electricity, and refined liquids
</commit_message>
<xml_diff>
--- a/gcam-data-system/energy-data/assumptions/Tables_A20s.xlsx
+++ b/gcam-data-system/energy-data/assumptions/Tables_A20s.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="23416"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <bookViews>
-    <workbookView xWindow="22720" yWindow="1240" windowWidth="24980" windowHeight="16240" tabRatio="684" firstSheet="14" activeTab="15"/>
+    <workbookView xWindow="240" yWindow="240" windowWidth="25360" windowHeight="15820" tabRatio="684" firstSheet="52" activeTab="54"/>
   </bookViews>
   <sheets>
     <sheet name="A21.sector.csv" sheetId="5" r:id="rId1"/>
@@ -21202,16 +21202,16 @@
         <v>57</v>
       </c>
       <c r="E7">
-        <v>1.25</v>
+        <v>0</v>
       </c>
       <c r="F7">
-        <v>1.25</v>
+        <v>0</v>
       </c>
       <c r="G7">
-        <v>1.25</v>
+        <v>0</v>
       </c>
       <c r="H7">
-        <v>1.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -21358,16 +21358,16 @@
         <v>57</v>
       </c>
       <c r="E13">
-        <v>1.1000000000000001</v>
+        <v>1.25</v>
       </c>
       <c r="F13">
-        <v>1.1000000000000001</v>
+        <v>1.25</v>
       </c>
       <c r="G13">
-        <v>1.1000000000000001</v>
+        <v>1.25</v>
       </c>
       <c r="H13">
-        <v>1.1000000000000001</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -21384,16 +21384,16 @@
         <v>57</v>
       </c>
       <c r="E14">
-        <v>0</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="F14">
-        <v>0</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="G14">
-        <v>0</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="H14">
-        <v>0</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="15" spans="1:8">

</xml_diff>